<commit_message>
Se adiciona nuevas funcionalidades
</commit_message>
<xml_diff>
--- a/ventas_dia2.xlsx
+++ b/ventas_dia2.xlsx
@@ -1,87 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-20610" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
-</file>
-
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="13">
-  <si>
-    <t>FechaVenta</t>
-  </si>
-  <si>
-    <t>Producto</t>
-  </si>
-  <si>
-    <t>PrecioVenta</t>
-  </si>
-  <si>
-    <t>Costo</t>
-  </si>
-  <si>
-    <t>Zona</t>
-  </si>
-  <si>
-    <t>Camisa</t>
-  </si>
-  <si>
-    <t>Pantalón</t>
-  </si>
-  <si>
-    <t>Zapatos</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Pantalón </t>
-  </si>
-  <si>
-    <t>CAMISA</t>
-  </si>
-  <si>
-    <t>Norte</t>
-  </si>
-  <si>
-    <t>Sur</t>
-  </si>
-  <si>
-    <t>Centro</t>
-  </si>
-</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -115,24 +71,105 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="VentasTabla" displayName="VentasTabla" ref="A1:E11" headerRowCount="1">
+  <autoFilter ref="A1:E11"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="FechaVenta"/>
+    <tableColumn id="2" name="Producto"/>
+    <tableColumn id="3" name="PrecioVenta"/>
+    <tableColumn id="4" name="Costo"/>
+    <tableColumn id="5" name="Zona"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -170,7 +207,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -204,6 +241,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -238,9 +276,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -413,192 +452,248 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <cols>
+    <col width="18.140625" bestFit="1" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" s="2">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FechaVenta</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>PrecioVenta</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Costo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
         <v>45099</v>
       </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Camisa</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>50000</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>30000</v>
       </c>
-      <c r="E2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="2">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
         <v>44974</v>
       </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3">
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Pantalón</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
         <v>80000</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>50000</v>
       </c>
-      <c r="E3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" s="2">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
         <v>45044</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>60000</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>40000</v>
       </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" s="2">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Centro</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
         <v>44994</v>
       </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Camisa</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
         <v>50000</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>30000</v>
       </c>
-      <c r="E5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" s="2">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
         <v>45030</v>
       </c>
-      <c r="B6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Zapatos</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
         <v>120000</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>80000</v>
       </c>
-      <c r="E6" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" s="2">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
         <v>44936</v>
       </c>
-      <c r="B7" t="s">
-        <v>8</v>
-      </c>
-      <c r="C7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Pantalón </t>
+        </is>
+      </c>
+      <c r="C7" t="n">
         <v>80000</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>50000</v>
       </c>
-      <c r="E7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" s="2">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
         <v>44948</v>
       </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Zapatos</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
         <v>120000</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>80000</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
-      <c r="A9" s="2">
+    <row r="9">
+      <c r="A9" s="2" t="n">
         <v>44963</v>
       </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CAMISA</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
         <v>50000</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>30000</v>
       </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" s="2">
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Centro</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
         <v>45014</v>
       </c>
-      <c r="B10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Zapatos</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
         <v>120000</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>80000</v>
       </c>
-      <c r="E10" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" s="2">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
         <v>44997</v>
       </c>
-      <c r="B11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Camisa</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
         <v>50000</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>30000</v>
       </c>
-      <c r="E11" t="s">
-        <v>12</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Centro</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>